<commit_message>
fix: Plusieurs modules, voici les recaps : - 6 fixes appliqués sur le module import : historique auto-refresh, calendrier EDT dynamique,   sauvegarde bâtiment/capacité salle, colonne Email parent, loading animé école, et bug   upsertedScheduleIds. Typecheck et lint passent — il reste à tester manuellement en lançant l'app.   (disable recaps in /config) - Module validations : historique filtrable ajouté aux onglets "Heures à valider" et   "Présences suspectes", notifications SMS/email scan de fin corrigées, bug page blanche résolu. Prêt    à tester en dev. (disable recaps in /config) - module attendance scan de fin : Qr de fin est maintenant toujours comparé au Qr de la salle de début de cours, pas à la sallle prévue.  pour s'assurer que le cours a été donné du début à la fin dans la même salle.
</commit_message>
<xml_diff>
--- a/templates/students.xlsx
+++ b/templates/students.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,9 +424,12 @@
         <v>Téléphone parent</v>
       </c>
       <c r="H1" t="str">
+        <v>Email parent</v>
+      </c>
+      <c r="I1" t="str">
         <v>Nom parent 2</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Téléphone parent 2</v>
       </c>
     </row>
@@ -453,15 +456,18 @@
         <v>2250701020304</v>
       </c>
       <c r="H2" t="str">
+        <v>parent@exemple.com</v>
+      </c>
+      <c r="I2" t="str">
         <v>Parent 2</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>2250506070809</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>